<commit_message>
Update with canonical TATA
</commit_message>
<xml_diff>
--- a/Supplemental Files/Table S3.xlsx
+++ b/Supplemental Files/Table S3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Šimon Pavlů\Desktop\2. Differencial analysis of barley promoterome\Supplement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADD77393-97FB-4548-96E1-C22AF507F408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F186714-BA58-48C4-8D44-2886A47CB28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,13 +660,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="4">
-        <v>580</v>
+        <v>19</v>
       </c>
       <c r="C3" s="4">
-        <v>1015</v>
+        <v>305</v>
       </c>
       <c r="D3" s="4">
-        <v>536</v>
+        <v>1805</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="16.2" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>